<commit_message>
docs: logged prompt and agent response for mutation tests
</commit_message>
<xml_diff>
--- a/data/ecs.xlsx
+++ b/data/ecs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/UST914/Desktop/blg-475-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9CE5DA-3289-904B-9F35-F3A679545A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAA1E87-8DEF-E84F-9B42-75115B9172B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="21000" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1803" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1808" uniqueCount="443">
   <si>
     <t>Type</t>
   </si>
@@ -2834,6 +2834,21 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>- Total equivalence classes: 296</t>
+  </si>
+  <si>
+    <t>- Covered by base tests: 109 / 296 = 36.82%</t>
+  </si>
+  <si>
+    <t>- Covered by mutated tests: 241 / 296 = 81.42%</t>
+  </si>
+  <si>
+    <t>- Improvement: +132 ECs = +44.60 percentage points</t>
+  </si>
+  <si>
+    <t>- Still uncovered after mutation: 55 / 296 = 18.58%</t>
   </si>
 </sst>
 </file>
@@ -2843,7 +2858,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2875,13 +2890,6 @@
       <color theme="1"/>
       <name val="Menlo"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4187,10 +4195,13 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA593DA-B4E3-4349-9AE3-137E67A4A1FB}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>358</v>
       </c>
@@ -4203,8 +4214,11 @@
       <c r="D1" s="6" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="F1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>361</v>
       </c>
@@ -4217,8 +4231,11 @@
       <c r="D2" s="7">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>362</v>
       </c>
@@ -4231,8 +4248,11 @@
       <c r="D3" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>363</v>
       </c>
@@ -4245,8 +4265,11 @@
       <c r="D4" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>364</v>
       </c>
@@ -4259,8 +4282,11 @@
       <c r="D5" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>365</v>
       </c>
@@ -4274,7 +4300,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>366</v>
       </c>
@@ -4288,7 +4314,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>367</v>
       </c>
@@ -4302,7 +4328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>368</v>
       </c>
@@ -4316,7 +4342,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>369</v>
       </c>
@@ -4330,7 +4356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>370</v>
       </c>
@@ -4344,7 +4370,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>371</v>
       </c>
@@ -4358,7 +4384,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>372</v>
       </c>
@@ -4372,7 +4398,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>373</v>
       </c>
@@ -4386,7 +4412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>374</v>
       </c>
@@ -4400,7 +4426,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>375</v>
       </c>

</xml_diff>